<commit_message>
Add experiment browser controls and per-step bias settings
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/templete_exel/different flows.xlsx
+++ b/templete_exel/different flows.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\PycharmProjects\FluidicControlSystem\templete_exel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1F19BE-A71D-4F31-98C7-80D5D2DA90C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785D73A1-0EA3-4044-8999-322251F74EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="8">
   <si>
     <t>Step</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>current</t>
+  </si>
+  <si>
+    <t>voltage</t>
   </si>
 </sst>
 </file>
@@ -441,13 +444,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C2">
-        <v>1.4</v>
+        <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
         <v>5</v>
@@ -458,13 +461,13 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C3">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
@@ -475,13 +478,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C4">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
         <v>5</v>
@@ -492,13 +495,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C5">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
         <v>5</v>
@@ -509,13 +512,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
         <v>5</v>
@@ -526,13 +529,13 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C7">
-        <v>2.2000000000000002</v>
+        <v>0.2</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
         <v>5</v>
@@ -543,10 +546,10 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C8">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="D8" t="s">
         <v>6</v>
@@ -560,10 +563,10 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C9">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -577,10 +580,10 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C10">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="s">
         <v>6</v>
@@ -594,10 +597,10 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C11">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
         <v>6</v>
@@ -611,10 +614,10 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="s">
         <v>6</v>
@@ -628,10 +631,10 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>420</v>
+        <v>300</v>
       </c>
       <c r="C13">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="D13" t="s">
         <v>6</v>

</xml_diff>